<commit_message>
Tidying up documentation files
</commit_message>
<xml_diff>
--- a/documentation/SimPaths_lag_structure_ES.xlsx
+++ b/documentation/SimPaths_lag_structure_ES.xlsx
@@ -1147,7 +1147,7 @@
     <t>schedule_check</t>
   </si>
   <si>
-    <t>Timing audit of every (model, covariate) pair that uses a current-period value (lag = c), comparing the position in the yearly schedule of the step that runs the model with the step that produces the covariate. Positions follow documentation/SimPathsEU_ScheduleNEW.xlsx (Order EU), with the order inside a step where it matters (H1 before H2; W1*-sel before W1*; I1a/I1b before labour supply). Flags: CHECK = producer runs later, so the c value still holds last year's value; same step = producer and consumer in the same step; OK = producer runs earlier; exogenous = not produced by a behavioural process (age, gender, region, macro, pension age); choice-specific = evaluated for each hours alternative inside the labour-supply step.</t>
+    <t>Timing audit of every (model, covariate) pair that uses a current-period value (lag = c), comparing the position in the yearly schedule of the step that runs the model with the step that produces the covariate. Positions follow documentation/SimPathsEU_Schedule.xlsx (Order EU), with the order inside a step where it matters (H1 before H2; W1*-sel before W1*; I1a/I1b before labour supply). Flags: CHECK = producer runs later, so the c value still holds last year's value; same step = producer and consumer in the same step; OK = producer runs earlier; exogenous = not produced by a behavioural process (age, gender, region, macro, pension age); choice-specific = evaluated for each hours alternative inside the labour-supply step.</t>
   </si>
   <si>
     <t>notes</t>
@@ -1327,7 +1327,7 @@
     <t>Schedule vs. lag-usage check</t>
   </si>
   <si>
-    <t>Shows every (process, covariate) pair where a current-period value (lag = c) is used. The flag compares the schedule position (Order EU in documentation/SimPathsEU_ScheduleNEW.xlsx) of the step running the model with that of the step producing the covariate.</t>
+    <t>Shows every (process, covariate) pair where a current-period value (lag = c) is used. The flag compares the schedule position (Order EU in documentation/SimPathsEU_Schedule.xlsx) of the step running the model with that of the step producing the covariate.</t>
   </si>
   <si>
     <t>Flag meanings:   CHECK = producer runs AFTER consumer (c still holds last year's value);   same step = producer and consumer at the same schedule position;   OK = producer runs before consumer;   exogenous = not produced by any behavioural process;   choice-specific = evaluated per hours alternative in the labour-supply step.</t>

</xml_diff>